<commit_message>
Use Hebrew cup serving for Muller yogurt
</commit_message>
<xml_diff>
--- a/data/source/foods.xlsx
+++ b/data/source/foods.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="R43b6526ecbbc47c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="R3f27c22332504ed5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20912,10 +20912,10 @@
         <x:v>יוגורטים ומעדנים</x:v>
       </x:c>
       <x:c r="C344" t="str">
-        <x:v>Müller 25g Protein Yogurt</x:v>
+        <x:v>יוגורט חלבון מולר 25 גרם חלבון</x:v>
       </x:c>
       <x:c r="D344" t="str">
-        <x:v>Müller</x:v>
+        <x:v>מולר</x:v>
       </x:c>
       <x:c r="E344" t="n">
         <x:v>200</x:v>
@@ -20940,7 +20940,7 @@
       <x:c r="M344"/>
       <x:c r="N344"/>
       <x:c r="O344" t="str">
-        <x:v>ל-100 גרם</x:v>
+        <x:v>גביע 200 גרם</x:v>
       </x:c>
       <x:c r="P344" t="str">
         <x:v>ממתין לבדיקה</x:v>
@@ -20976,7 +20976,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe8fbd646de94eb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re290cd4c764541cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Use 200g cup servings for Yoplait GO
</commit_message>
<xml_diff>
--- a/data/source/foods.xlsx
+++ b/data/source/foods.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="R3f27c22332504ed5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="R9c03438ab9334abe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5162,8 +5162,8 @@
       <x:c r="E35" s="12">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="F35" s="12" t="s">
-        <x:v>24</x:v>
+      <x:c r="F35" s="12" t="str">
+        <x:v>גביע</x:v>
       </x:c>
       <x:c r="G35" s="11">
         <x:v>72</x:v>
@@ -5189,15 +5189,26 @@
       <x:c r="N35" s="14" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="O35" s="15" t="s">
-        <x:v>26</x:v>
+      <x:c r="O35" s="15" t="str">
+        <x:v>גביע 200 גרם</x:v>
       </x:c>
       <x:c r="P35" s="15" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="Q35" s="15"/>
+      <x:c r="Q35" s="15" t="str">
+        <x:v>גביע אחד של 200 גרם; סה״כ לגביע: 144 קלוריות, 20 גרם חלבון, 7 גרם פחמימות ו-4 גרם שומן</x:v>
+      </x:c>
       <x:c r="R35" s="16" t="s">
         <x:v>127</x:v>
+      </x:c>
+      <x:c r="S35" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T35" t="n">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="U35" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="24" customHeight="1">
@@ -5216,8 +5227,8 @@
       <x:c r="E36" s="12">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="F36" s="12" t="s">
-        <x:v>24</x:v>
+      <x:c r="F36" s="12" t="str">
+        <x:v>גביע</x:v>
       </x:c>
       <x:c r="G36" s="11">
         <x:v>86</x:v>
@@ -5243,15 +5254,26 @@
       <x:c r="N36" s="14" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="O36" s="15" t="s">
-        <x:v>26</x:v>
+      <x:c r="O36" s="15" t="str">
+        <x:v>גביע 200 גרם</x:v>
       </x:c>
       <x:c r="P36" s="15" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="Q36" s="15"/>
+      <x:c r="Q36" s="15" t="str">
+        <x:v>גביע אחד של 200 גרם; סה״כ לגביע: 172 קלוריות, 25 גרם חלבון, 8.8 גרם פחמימות ו-4 גרם שומן</x:v>
+      </x:c>
       <x:c r="R36" s="16" t="s">
         <x:v>130</x:v>
+      </x:c>
+      <x:c r="S36" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T36" t="n">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="U36" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="24" customHeight="1">
@@ -20976,7 +20998,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re290cd4c764541cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc650d19148c24cda"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Danone PRO yogurt example
</commit_message>
<xml_diff>
--- a/data/source/foods.xlsx
+++ b/data/source/foods.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="R9c03438ab9334abe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="Rd9437cc4d96049b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3178,7 +3178,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FoodBlock01" displayName="FoodBlock01" ref="A4:R343" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FoodBlock01" displayName="FoodBlock01" ref="A4:R344" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="מס׳"/>
     <x:tableColumn id="2" name="קטגוריה"/>
@@ -3421,7 +3421,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="27" t="str">
-        <x:v>מאגר מזונות ישראלי | 340 מוצרים</x:v>
+        <x:v>מאגר מזונות ישראלי | 341 מוצרים</x:v>
       </x:c>
       <x:c r="B1" s="27"/>
       <x:c r="C1" s="27"/>
@@ -3443,7 +3443,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="28" t="str">
-        <x:v>מוצרים 317–340: מאפים, מנות מוכנות ומוצרים ממותגים.</x:v>
+        <x:v>מוצר 341: דנונה PRO טבעי 1.5%, ערכים לגביע 200 גרם.</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
       <x:c r="C2" s="28"/>
@@ -20981,6 +20981,69 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="345">
+      <x:c r="A345" t="n">
+        <x:v>341</x:v>
+      </x:c>
+      <x:c r="B345" t="str">
+        <x:v>יוגורטים ומעדנים</x:v>
+      </x:c>
+      <x:c r="C345" t="str">
+        <x:v>דנונה PRO יוגורט 20 גרם חלבון 1.5% שומן</x:v>
+      </x:c>
+      <x:c r="D345" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E345" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F345" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G345" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="H345" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I345" t="n">
+        <x:v>3.4</x:v>
+      </x:c>
+      <x:c r="J345" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="K345" t="n">
+        <x:v>3.4</x:v>
+      </x:c>
+      <x:c r="L345" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M345" t="n">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="N345"/>
+      <x:c r="O345" t="str">
+        <x:v>גביע 200 גרם</x:v>
+      </x:c>
+      <x:c r="P345" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q345" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 140 קלוריות, 20 גרם חלבון, 6.8 גרם פחמימות, 3 גרם שומן, 6.8 גרם סוכרים, 70 מ״ג נתרן ו-198 מ״ג סידן.</x:v>
+      </x:c>
+      <x:c r="R345" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S345" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T345" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="U345" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:R1"/>
@@ -20998,7 +21061,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc650d19148c24cda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0333e5bbd9544b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix workout rotation and publish current app updates
</commit_message>
<xml_diff>
--- a/data/source/foods.xlsx
+++ b/data/source/foods.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="R9c03438ab9334abe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="Rd9437cc4d96049b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3178,7 +3178,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FoodBlock01" displayName="FoodBlock01" ref="A4:R343" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FoodBlock01" displayName="FoodBlock01" ref="A4:R344" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="מס׳"/>
     <x:tableColumn id="2" name="קטגוריה"/>
@@ -3421,7 +3421,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="27" t="str">
-        <x:v>מאגר מזונות ישראלי | 340 מוצרים</x:v>
+        <x:v>מאגר מזונות ישראלי | 341 מוצרים</x:v>
       </x:c>
       <x:c r="B1" s="27"/>
       <x:c r="C1" s="27"/>
@@ -3443,7 +3443,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="28" t="str">
-        <x:v>מוצרים 317–340: מאפים, מנות מוכנות ומוצרים ממותגים.</x:v>
+        <x:v>מוצר 341: דנונה PRO טבעי 1.5%, ערכים לגביע 200 גרם.</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
       <x:c r="C2" s="28"/>
@@ -20981,6 +20981,69 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="345">
+      <x:c r="A345" t="n">
+        <x:v>341</x:v>
+      </x:c>
+      <x:c r="B345" t="str">
+        <x:v>יוגורטים ומעדנים</x:v>
+      </x:c>
+      <x:c r="C345" t="str">
+        <x:v>דנונה PRO יוגורט 20 גרם חלבון 1.5% שומן</x:v>
+      </x:c>
+      <x:c r="D345" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E345" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F345" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G345" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="H345" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I345" t="n">
+        <x:v>3.4</x:v>
+      </x:c>
+      <x:c r="J345" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="K345" t="n">
+        <x:v>3.4</x:v>
+      </x:c>
+      <x:c r="L345" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M345" t="n">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="N345"/>
+      <x:c r="O345" t="str">
+        <x:v>גביע 200 גרם</x:v>
+      </x:c>
+      <x:c r="P345" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q345" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 140 קלוריות, 20 גרם חלבון, 6.8 גרם פחמימות, 3 גרם שומן, 6.8 גרם סוכרים, 70 מ״ג נתרן ו-198 מ״ג סידן.</x:v>
+      </x:c>
+      <x:c r="R345" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S345" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T345" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="U345" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:R1"/>
@@ -20998,7 +21061,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc650d19148c24cda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0333e5bbd9544b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Reconcile production and restore progress averages
</commit_message>
<xml_diff>
--- a/data/source/foods.xlsx
+++ b/data/source/foods.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="Rd9437cc4d96049b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="Rec7313908b084976"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3178,7 +3178,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FoodBlock01" displayName="FoodBlock01" ref="A4:R344" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FoodBlock01" displayName="FoodBlock01" ref="A4:R363" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="מס׳"/>
     <x:tableColumn id="2" name="קטגוריה"/>
@@ -3421,7 +3421,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="27" t="str">
-        <x:v>מאגר מזונות ישראלי | 341 מוצרים</x:v>
+        <x:v>מאגר מזונות ישראלי | 359 מוצרים</x:v>
       </x:c>
       <x:c r="B1" s="27"/>
       <x:c r="C1" s="27"/>
@@ -3443,7 +3443,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="28" t="str">
-        <x:v>מוצר 341: דנונה PRO טבעי 1.5%, ערכים לגביע 200 גרם.</x:v>
+        <x:v>מוצר 359: קינוח בצק מטוגן במילוי קרם פטיסייר, ערכים ליחידה של 150 גרם.</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
       <x:c r="C2" s="28"/>
@@ -20986,10 +20986,10 @@
         <x:v>341</x:v>
       </x:c>
       <x:c r="B345" t="str">
-        <x:v>יוגורטים ומעדנים</x:v>
+        <x:v>יוגורט חלבון</x:v>
       </x:c>
       <x:c r="C345" t="str">
-        <x:v>דנונה PRO יוגורט 20 גרם חלבון 1.5% שומן</x:v>
+        <x:v>דנונה PRO יוגורט 20 גר׳ חלבון 1.5% שומן</x:v>
       </x:c>
       <x:c r="D345" t="str">
         <x:v>דנונה</x:v>
@@ -21041,6 +21041,1130 @@
         <x:v>140</x:v>
       </x:c>
       <x:c r="U345" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="346">
+      <x:c r="A346" t="n">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="B346" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C346" t="str">
+        <x:v>דנונה PRO יוגורט שכבות בטעם מנגו 20 גר׳ חלבון 0% שומן</x:v>
+      </x:c>
+      <x:c r="D346" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E346" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="F346" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G346" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="H346" t="n">
+        <x:v>9.3</x:v>
+      </x:c>
+      <x:c r="I346" t="n">
+        <x:v>3.9</x:v>
+      </x:c>
+      <x:c r="J346" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K346" t="n">
+        <x:v>3.6</x:v>
+      </x:c>
+      <x:c r="L346" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="M346" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="N346"/>
+      <x:c r="O346" t="str">
+        <x:v>גביע 215 גרם</x:v>
+      </x:c>
+      <x:c r="P346" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q346" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 120.4 קלוריות ו-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R346" t="str">
+        <x:v>https://danone.strauss-group.com/products/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro-%d7%99%d7%95%d7%92%d7%95%d7%a8%d7%98-%d7%a9%d7%9b%d7%91%d7%95%d7%aa-%d7%91%d7%98%d7%a2%d7%9d-%d7%9e%d7%a0%d7%92%d7%95-20-%d7%92%d7%a8%d7%b3-%d7%97%d7%9c%d7%91%d7%95/</x:v>
+      </x:c>
+      <x:c r="S346" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="T346" t="n">
+        <x:v>120.4</x:v>
+      </x:c>
+      <x:c r="U346" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="347">
+      <x:c r="A347" t="n">
+        <x:v>343</x:v>
+      </x:c>
+      <x:c r="B347" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C347" t="str">
+        <x:v>דנונה PRO יוגורט שכבות בטעם פירות יער 20 גר׳ חלבון 0% שומן</x:v>
+      </x:c>
+      <x:c r="D347" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E347" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="F347" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G347" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="H347" t="n">
+        <x:v>9.3</x:v>
+      </x:c>
+      <x:c r="I347" t="n">
+        <x:v>3.7</x:v>
+      </x:c>
+      <x:c r="J347" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K347" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="L347" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="M347" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="N347"/>
+      <x:c r="O347" t="str">
+        <x:v>גביע 215 גרם</x:v>
+      </x:c>
+      <x:c r="P347" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q347" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 118.3 קלוריות ו-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R347" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S347" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="T347" t="n">
+        <x:v>118.3</x:v>
+      </x:c>
+      <x:c r="U347" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="348">
+      <x:c r="A348" t="n">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="B348" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C348" t="str">
+        <x:v>דנונה PRO יוגורט קראנצ' בטעם מתיקות מעודנת עם פתיתי סויה מצופים שוקולד מריר 20 גר׳ חלבון 3.9% שומן</x:v>
+      </x:c>
+      <x:c r="D348" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E348" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="F348" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G348" t="n">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="H348" t="n">
+        <x:v>11.2</x:v>
+      </x:c>
+      <x:c r="I348" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J348" t="n">
+        <x:v>3.9</x:v>
+      </x:c>
+      <x:c r="K348" t="n">
+        <x:v>7.7</x:v>
+      </x:c>
+      <x:c r="L348" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="M348" t="n">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="N348"/>
+      <x:c r="O348" t="str">
+        <x:v>גביע 180 גרם</x:v>
+      </x:c>
+      <x:c r="P348" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q348" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 217.8 קלוריות וכ-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R348" t="str">
+        <x:v>https://danone.strauss-group.com/products/%d7%a4%d7%a8%d7%95-%d7%a7%d7%a8%d7%90%d7%a0%d7%a6-%d7%a9%d7%95%d7%a7%d7%95%d7%9c%d7%93-%d7%9e%d7%a8%d7%99%d7%a8/</x:v>
+      </x:c>
+      <x:c r="S348" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="T348" t="n">
+        <x:v>217.8</x:v>
+      </x:c>
+      <x:c r="U348" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="349">
+      <x:c r="A349" t="n">
+        <x:v>345</x:v>
+      </x:c>
+      <x:c r="B349" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C349" t="str">
+        <x:v>דנונה PRO יוגורט ללא סוכר 25 גר׳ חלבון 2% שומן</x:v>
+      </x:c>
+      <x:c r="D349" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E349" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="F349" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G349" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="H349" t="n">
+        <x:v>11.6</x:v>
+      </x:c>
+      <x:c r="I349" t="n">
+        <x:v>4.1</x:v>
+      </x:c>
+      <x:c r="J349" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K349" t="n">
+        <x:v>3.9</x:v>
+      </x:c>
+      <x:c r="L349" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="M349" t="n">
+        <x:v>314</x:v>
+      </x:c>
+      <x:c r="N349"/>
+      <x:c r="O349" t="str">
+        <x:v>גביע 215 גרם</x:v>
+      </x:c>
+      <x:c r="P349" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q349" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 189.2 קלוריות וכ-25 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R349" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S349" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="T349" t="n">
+        <x:v>189.2</x:v>
+      </x:c>
+      <x:c r="U349" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="350">
+      <x:c r="A350" t="n">
+        <x:v>346</x:v>
+      </x:c>
+      <x:c r="B350" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C350" t="str">
+        <x:v>דנונה PRO יוגורט בטעם וניל ללא סוכר 25 גר׳ חלבון 2% שומן</x:v>
+      </x:c>
+      <x:c r="D350" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E350" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="F350" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G350" t="n">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="H350" t="n">
+        <x:v>11.6</x:v>
+      </x:c>
+      <x:c r="I350" t="n">
+        <x:v>4.3</x:v>
+      </x:c>
+      <x:c r="J350" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K350" t="n">
+        <x:v>3.9</x:v>
+      </x:c>
+      <x:c r="L350" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="M350" t="n">
+        <x:v>314</x:v>
+      </x:c>
+      <x:c r="N350"/>
+      <x:c r="O350" t="str">
+        <x:v>גביע 215 גרם</x:v>
+      </x:c>
+      <x:c r="P350" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q350" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 191.4 קלוריות וכ-25 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R350" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S350" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="T350" t="n">
+        <x:v>191.4</x:v>
+      </x:c>
+      <x:c r="U350" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="351">
+      <x:c r="A351" t="n">
+        <x:v>347</x:v>
+      </x:c>
+      <x:c r="B351" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C351" t="str">
+        <x:v>דנונה PRO בטעם קרם לימון ללא סוכר 20 גר׳ חלבון 0% שומן</x:v>
+      </x:c>
+      <x:c r="D351" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E351" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F351" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G351" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="H351" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I351" t="n">
+        <x:v>3.4</x:v>
+      </x:c>
+      <x:c r="J351" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K351" t="n">
+        <x:v>3.2</x:v>
+      </x:c>
+      <x:c r="L351" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="M351" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="N351"/>
+      <x:c r="O351" t="str">
+        <x:v>גביע 200 גרם</x:v>
+      </x:c>
+      <x:c r="P351" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q351" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 110 קלוריות ו-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R351" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S351" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T351" t="n">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="U351" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="352">
+      <x:c r="A352" t="n">
+        <x:v>348</x:v>
+      </x:c>
+      <x:c r="B352" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C352" t="str">
+        <x:v>דנונה PRO יוגורט קראנצ' בטעם מתיקות מעודנת עם פתיתי סויה מצופים שוקולד חלב 20 גר׳ חלבון 3.7% שומן</x:v>
+      </x:c>
+      <x:c r="D352" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E352" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="F352" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G352" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="H352" t="n">
+        <x:v>11.2</x:v>
+      </x:c>
+      <x:c r="I352" t="n">
+        <x:v>8.7</x:v>
+      </x:c>
+      <x:c r="J352" t="n">
+        <x:v>3.7</x:v>
+      </x:c>
+      <x:c r="K352" t="n">
+        <x:v>8.4</x:v>
+      </x:c>
+      <x:c r="L352" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="M352" t="n">
+        <x:v>227</x:v>
+      </x:c>
+      <x:c r="N352"/>
+      <x:c r="O352" t="str">
+        <x:v>גביע 180 גרם</x:v>
+      </x:c>
+      <x:c r="P352" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q352" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 216 קלוריות וכ-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R352" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S352" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="T352" t="n">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="U352" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="353">
+      <x:c r="A353" t="n">
+        <x:v>349</x:v>
+      </x:c>
+      <x:c r="B353" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C353" t="str">
+        <x:v>דנונה PRO יוגורט בטעם רול קינמון ללא סוכר 20 גר׳ חלבון 0% שומן</x:v>
+      </x:c>
+      <x:c r="D353" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E353" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F353" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G353" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="H353" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I353" t="n">
+        <x:v>3.4</x:v>
+      </x:c>
+      <x:c r="J353" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K353" t="n">
+        <x:v>3.2</x:v>
+      </x:c>
+      <x:c r="L353" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="M353" t="n">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="N353"/>
+      <x:c r="O353" t="str">
+        <x:v>גביע 200 גרם</x:v>
+      </x:c>
+      <x:c r="P353" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q353" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 112 קלוריות ו-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R353" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S353" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T353" t="n">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="U353" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="354">
+      <x:c r="A354" t="n">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="B354" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C354" t="str">
+        <x:v>דנונה PRO משקה יוגורט בטעם וניל עוגיות 20 גר׳ חלבון 1% שומן</x:v>
+      </x:c>
+      <x:c r="D354" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E354" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="F354" t="str">
+        <x:v>בקבוק</x:v>
+      </x:c>
+      <x:c r="G354" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="H354" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I354" t="n">
+        <x:v>4.2</x:v>
+      </x:c>
+      <x:c r="J354" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K354" t="n">
+        <x:v>3.6</x:v>
+      </x:c>
+      <x:c r="L354" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="M354" t="n">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="N354"/>
+      <x:c r="O354" t="str">
+        <x:v>בקבוק 250 מ״ל</x:v>
+      </x:c>
+      <x:c r="P354" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q354" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לבקבוק: 152.5 קלוריות ו-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R354" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S354" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T354" t="n">
+        <x:v>152.5</x:v>
+      </x:c>
+      <x:c r="U354" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="355">
+      <x:c r="A355" t="n">
+        <x:v>351</x:v>
+      </x:c>
+      <x:c r="B355" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C355" t="str">
+        <x:v>דנונה PRO בטעם וניל עוגיות ללא סוכר 20 גר׳ חלבון 0% שומן</x:v>
+      </x:c>
+      <x:c r="D355" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E355" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F355" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G355" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="H355" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I355" t="n">
+        <x:v>3.4</x:v>
+      </x:c>
+      <x:c r="J355" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K355" t="n">
+        <x:v>3.2</x:v>
+      </x:c>
+      <x:c r="L355" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="M355" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="N355"/>
+      <x:c r="O355" t="str">
+        <x:v>גביע 200 גרם</x:v>
+      </x:c>
+      <x:c r="P355" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q355" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 112 קלוריות ו-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R355" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S355" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T355" t="n">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="U355" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="356">
+      <x:c r="A356" t="n">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="B356" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C356" t="str">
+        <x:v>דנונה PRO יוגורט בטעם בננה טופי ללא סוכר 20 גר׳ חלבון 0% שומן</x:v>
+      </x:c>
+      <x:c r="D356" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E356" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F356" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G356" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="H356" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I356" t="n">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="J356" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K356" t="n">
+        <x:v>3.2</x:v>
+      </x:c>
+      <x:c r="L356" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="M356" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="N356"/>
+      <x:c r="O356" t="str">
+        <x:v>גביע 200 גרם</x:v>
+      </x:c>
+      <x:c r="P356" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q356" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 112 קלוריות ו-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R356" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S356" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T356" t="n">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="U356" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="357">
+      <x:c r="A357" t="n">
+        <x:v>353</x:v>
+      </x:c>
+      <x:c r="B357" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C357" t="str">
+        <x:v>דנונה PRO יוגורט בטעם פיסטוק ללא סוכר 20 גר׳ חלבון 0% שומן</x:v>
+      </x:c>
+      <x:c r="D357" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E357" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F357" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G357" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="H357" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I357" t="n">
+        <x:v>3.4</x:v>
+      </x:c>
+      <x:c r="J357" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K357" t="n">
+        <x:v>3.2</x:v>
+      </x:c>
+      <x:c r="L357" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="M357" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="N357"/>
+      <x:c r="O357" t="str">
+        <x:v>גביע 200 גרם</x:v>
+      </x:c>
+      <x:c r="P357" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q357" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 110 קלוריות ו-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R357" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S357" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T357" t="n">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="U357" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="358">
+      <x:c r="A358" t="n">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="B358" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C358" t="str">
+        <x:v>דנונה PRO משקה יוגורט בטעם תות ללא סוכר 20 גר׳ חלבון 1% שומן</x:v>
+      </x:c>
+      <x:c r="D358" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E358" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="F358" t="str">
+        <x:v>בקבוק</x:v>
+      </x:c>
+      <x:c r="G358" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="H358" t="n">
+        <x:v>7.9</x:v>
+      </x:c>
+      <x:c r="I358" t="n">
+        <x:v>3.9</x:v>
+      </x:c>
+      <x:c r="J358" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K358" t="n">
+        <x:v>3.4</x:v>
+      </x:c>
+      <x:c r="L358" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="M358" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="N358"/>
+      <x:c r="O358" t="str">
+        <x:v>בקבוק 250 מ״ל</x:v>
+      </x:c>
+      <x:c r="P358" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q358" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לבקבוק: 147.5 קלוריות וכ-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R358" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S358" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T358" t="n">
+        <x:v>147.5</x:v>
+      </x:c>
+      <x:c r="U358" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="359">
+      <x:c r="A359" t="n">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="B359" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C359" t="str">
+        <x:v>דנונה PRO יוגורט 21 גר׳ חלבון 0% שומן</x:v>
+      </x:c>
+      <x:c r="D359" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E359" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F359" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G359" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="H359" t="n">
+        <x:v>10.5</x:v>
+      </x:c>
+      <x:c r="I359" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="J359" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K359" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="L359" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="M359" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N359"/>
+      <x:c r="O359" t="str">
+        <x:v>גביע 200 גרם</x:v>
+      </x:c>
+      <x:c r="P359" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q359" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 116 קלוריות ו-21 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R359" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S359" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T359" t="n">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="U359" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="360">
+      <x:c r="A360" t="n">
+        <x:v>356</x:v>
+      </x:c>
+      <x:c r="B360" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C360" t="str">
+        <x:v>דנונה PRO יוגורט בטעם וניל 20 גר׳ חלבון 0% שומן</x:v>
+      </x:c>
+      <x:c r="D360" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E360" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F360" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G360" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="H360" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I360" t="n">
+        <x:v>5.6</x:v>
+      </x:c>
+      <x:c r="J360" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K360" t="n">
+        <x:v>5.6</x:v>
+      </x:c>
+      <x:c r="L360" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="M360" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="N360"/>
+      <x:c r="O360" t="str">
+        <x:v>גביע 200 גרם</x:v>
+      </x:c>
+      <x:c r="P360" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q360" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 130 קלוריות ו-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R360" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S360" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T360" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="U360" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="361">
+      <x:c r="A361" t="n">
+        <x:v>357</x:v>
+      </x:c>
+      <x:c r="B361" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C361" t="str">
+        <x:v>דנונה PRO יוגורט בטעם פירות יער 20 גר׳ חלבון 0% שומן</x:v>
+      </x:c>
+      <x:c r="D361" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E361" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F361" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G361" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="H361" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I361" t="n">
+        <x:v>5.6</x:v>
+      </x:c>
+      <x:c r="J361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K361" t="n">
+        <x:v>5.6</x:v>
+      </x:c>
+      <x:c r="L361" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="M361" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="N361"/>
+      <x:c r="O361" t="str">
+        <x:v>גביע 200 גרם</x:v>
+      </x:c>
+      <x:c r="P361" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q361" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 130 קלוריות ו-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R361" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S361" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T361" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="U361" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="362">
+      <x:c r="A362" t="n">
+        <x:v>358</x:v>
+      </x:c>
+      <x:c r="B362" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C362" t="str">
+        <x:v>דנונה PRO יוגורט בטעם תות 20 גר׳ חלבון 0% שומן</x:v>
+      </x:c>
+      <x:c r="D362" t="str">
+        <x:v>דנונה</x:v>
+      </x:c>
+      <x:c r="E362" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F362" t="str">
+        <x:v>גביע</x:v>
+      </x:c>
+      <x:c r="G362" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="H362" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I362" t="n">
+        <x:v>5.6</x:v>
+      </x:c>
+      <x:c r="J362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K362" t="n">
+        <x:v>5.6</x:v>
+      </x:c>
+      <x:c r="L362" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="M362" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="N362"/>
+      <x:c r="O362" t="str">
+        <x:v>גביע 200 גרם</x:v>
+      </x:c>
+      <x:c r="P362" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q362" t="str">
+        <x:v>ערכים ל-100 גרם לפי דנונה; סה״כ לגביע: 130 קלוריות ו-20 גרם חלבון.</x:v>
+      </x:c>
+      <x:c r="R362" t="str">
+        <x:v>https://danone.strauss-group.com/product/%d7%93%d7%a0%d7%95%d7%a0%d7%94-pro/</x:v>
+      </x:c>
+      <x:c r="S362" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="T362" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="U362" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="363">
+      <x:c r="A363" t="n">
+        <x:v>359</x:v>
+      </x:c>
+      <x:c r="B363" t="str">
+        <x:v>מאפי מאפייה</x:v>
+      </x:c>
+      <x:c r="C363" t="str">
+        <x:v>קינוח בצק מטוגן במילוי קרם פטיסייר</x:v>
+      </x:c>
+      <x:c r="D363"/>
+      <x:c r="E363" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F363" t="str">
+        <x:v>יחידה</x:v>
+      </x:c>
+      <x:c r="G363" t="n">
+        <x:v>466.67</x:v>
+      </x:c>
+      <x:c r="H363" t="n">
+        <x:v>6.67</x:v>
+      </x:c>
+      <x:c r="I363" t="n">
+        <x:v>46.67</x:v>
+      </x:c>
+      <x:c r="J363" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="K363"/>
+      <x:c r="L363"/>
+      <x:c r="M363"/>
+      <x:c r="N363"/>
+      <x:c r="O363" t="str">
+        <x:v>יחידה 150 גרם</x:v>
+      </x:c>
+      <x:c r="P363" t="str">
+        <x:v>ממתין לבדיקה</x:v>
+      </x:c>
+      <x:c r="Q363" t="str">
+        <x:v>ערכים שנמסרו על ידי המשתמש; סה״כ ליחידה של 150 גרם: 700 קלוריות, 10 גרם חלבון, 70 גרם פחמימות ו-42 גרם שומן.</x:v>
+      </x:c>
+      <x:c r="R363"/>
+      <x:c r="S363" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="T363" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="U363" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -21061,7 +22185,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0333e5bbd9544b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11ae91d76ffd4260"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Muller vanilla protein drink
</commit_message>
<xml_diff>
--- a/data/source/foods.xlsx
+++ b/data/source/foods.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="Rec7313908b084976"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="Re1f3a855bae34bf5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2912,8 +2912,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="164" formatCode="0.0"/>
+    <x:numFmt numFmtId="200" formatCode="@"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -3060,7 +3061,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="29">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3136,6 +3137,7 @@
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -3421,7 +3423,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="27" t="str">
-        <x:v>מאגר מזונות ישראלי | 359 מוצרים</x:v>
+        <x:v>מאגר מזונות ישראלי | 360 מוצרים</x:v>
       </x:c>
       <x:c r="B1" s="27"/>
       <x:c r="C1" s="27"/>
@@ -3443,7 +3445,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="28" t="str">
-        <x:v>מוצר 359: קינוח בצק מטוגן במילוי קרם פטיסייר, ערכים ליחידה של 150 גרם.</x:v>
+        <x:v>מוצר 360: משקה חלבון מולר וניל 40 גרם חלבון 0% שומן, ערכים לבקבוק 350 מ״ל.</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
       <x:c r="C2" s="28"/>
@@ -22168,6 +22170,92 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="364">
+      <x:c r="A364" t="str">
+        <x:v>muller-protein-40-vanilla-350ml</x:v>
+      </x:c>
+      <x:c r="B364" t="str">
+        <x:v>יוגורט חלבון</x:v>
+      </x:c>
+      <x:c r="C364" t="str">
+        <x:v>משקה חלבון מולר וניל 40 גרם חלבון 0% שומן</x:v>
+      </x:c>
+      <x:c r="D364" t="str">
+        <x:v>מולר</x:v>
+      </x:c>
+      <x:c r="E364" t="n">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="F364" t="str">
+        <x:v>בקבוק</x:v>
+      </x:c>
+      <x:c r="G364" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="H364" t="n">
+        <x:v>11.43</x:v>
+      </x:c>
+      <x:c r="I364" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="J364" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K364" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="L364" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="M364" t="n">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="N364" s="29" t="str">
+        <x:v>7290114312551</x:v>
+      </x:c>
+      <x:c r="O364" t="str">
+        <x:v>בקבוק 350 מ״ל</x:v>
+      </x:c>
+      <x:c r="P364" t="str">
+        <x:v>מאושר</x:v>
+      </x:c>
+      <x:c r="Q364" t="str">
+        <x:v>ערכים ל-100 מ״ל לפי תווית המוצר; סה״כ לבקבוק 350 מ״ל: 224 קלוריות, 40 גרם חלבון, 15.75 גרם פחמימות ו-0 גרם שומן.</x:v>
+      </x:c>
+      <x:c r="R364"/>
+      <x:c r="S364" t="n">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="T364" t="n">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="U364" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="365">
+      <x:c r="A365"/>
+      <x:c r="B365"/>
+      <x:c r="C365"/>
+      <x:c r="D365"/>
+      <x:c r="E365"/>
+      <x:c r="F365"/>
+      <x:c r="G365"/>
+      <x:c r="H365"/>
+      <x:c r="I365"/>
+      <x:c r="J365"/>
+      <x:c r="K365"/>
+      <x:c r="L365"/>
+      <x:c r="M365"/>
+      <x:c r="N365"/>
+      <x:c r="O365"/>
+      <x:c r="P365"/>
+      <x:c r="Q365"/>
+      <x:c r="R365"/>
+      <x:c r="S365"/>
+      <x:c r="T365"/>
+      <x:c r="U365"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:R1"/>
@@ -22185,7 +22273,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11ae91d76ffd4260"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbefcf396fe214c65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add roasted cashews to food catalog
</commit_message>
<xml_diff>
--- a/data/source/foods.xlsx
+++ b/data/source/foods.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="Re1f3a855bae34bf5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="R2ee725917a884f96"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3423,7 +3423,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="27" t="str">
-        <x:v>מאגר מזונות ישראלי | 360 מוצרים</x:v>
+        <x:v>מאגר מזונות ישראלי | 361 מוצרים</x:v>
       </x:c>
       <x:c r="B1" s="27"/>
       <x:c r="C1" s="27"/>
@@ -3445,7 +3445,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="28" t="str">
-        <x:v>מוצר 360: משקה חלבון מולר וניל 40 גרם חלבון 0% שומן, ערכים לבקבוק 350 מ״ל.</x:v>
+        <x:v>מוצר 361: קשיו קלוי, ערכים ל-100 גרם לפי נתוני המשתמש.</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
       <x:c r="C2" s="28"/>
@@ -22234,23 +22234,45 @@
       </x:c>
     </x:row>
     <x:row r="365">
-      <x:c r="A365"/>
-      <x:c r="B365"/>
-      <x:c r="C365"/>
+      <x:c r="A365" t="str">
+        <x:v>roasted-cashews</x:v>
+      </x:c>
+      <x:c r="B365" t="str">
+        <x:v>אגוזים וזרעים</x:v>
+      </x:c>
+      <x:c r="C365" t="str">
+        <x:v>קשיו קלוי</x:v>
+      </x:c>
       <x:c r="D365"/>
       <x:c r="E365"/>
       <x:c r="F365"/>
-      <x:c r="G365"/>
-      <x:c r="H365"/>
-      <x:c r="I365"/>
-      <x:c r="J365"/>
+      <x:c r="G365" t="n">
+        <x:v>606</x:v>
+      </x:c>
+      <x:c r="H365" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="I365" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J365" t="n">
+        <x:v>47</x:v>
+      </x:c>
       <x:c r="K365"/>
-      <x:c r="L365"/>
+      <x:c r="L365" t="n">
+        <x:v>600</x:v>
+      </x:c>
       <x:c r="M365"/>
-      <x:c r="N365"/>
-      <x:c r="O365"/>
-      <x:c r="P365"/>
-      <x:c r="Q365"/>
+      <x:c r="N365" s="29"/>
+      <x:c r="O365" t="str">
+        <x:v>ל-100 גרם</x:v>
+      </x:c>
+      <x:c r="P365" t="str">
+        <x:v>ממתין לבדיקה</x:v>
+      </x:c>
+      <x:c r="Q365" t="str">
+        <x:v>ערכים ל-100 גרם שנמסרו על ידי המשתמש; הנתרן הוא ערך משוער של כ-600 מ״ג.</x:v>
+      </x:c>
       <x:c r="R365"/>
       <x:c r="S365"/>
       <x:c r="T365"/>
@@ -22273,7 +22295,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbefcf396fe214c65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f4d7261ae30498d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add walnuts and roasted salted almonds
</commit_message>
<xml_diff>
--- a/data/source/foods.xlsx
+++ b/data/source/foods.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="R2ee725917a884f96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="Rb0aab3d189e14df2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3423,7 +3423,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="27" t="str">
-        <x:v>מאגר מזונות ישראלי | 361 מוצרים</x:v>
+        <x:v>מאגר מזונות ישראלי | 363 מוצרים</x:v>
       </x:c>
       <x:c r="B1" s="27"/>
       <x:c r="C1" s="27"/>
@@ -3445,7 +3445,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="28" t="str">
-        <x:v>מוצר 361: קשיו קלוי, ערכים ל-100 גרם לפי נתוני המשתמש.</x:v>
+        <x:v>מוצרים 362–363: אגוזי מלך ושקדים קלויים ומלוחים, לפי נתוני המשתמש.</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
       <x:c r="C2" s="28"/>
@@ -22278,6 +22278,114 @@
       <x:c r="T365"/>
       <x:c r="U365"/>
     </x:row>
+    <x:row r="366">
+      <x:c r="A366" t="str">
+        <x:v>walnuts</x:v>
+      </x:c>
+      <x:c r="B366" t="str">
+        <x:v>אגוזים וזרעים</x:v>
+      </x:c>
+      <x:c r="C366" t="str">
+        <x:v>אגוזי מלך</x:v>
+      </x:c>
+      <x:c r="D366"/>
+      <x:c r="E366"/>
+      <x:c r="F366" t="str">
+        <x:v>יחידה</x:v>
+      </x:c>
+      <x:c r="G366" t="n">
+        <x:v>654</x:v>
+      </x:c>
+      <x:c r="H366" t="n">
+        <x:v>15.2</x:v>
+      </x:c>
+      <x:c r="I366" t="n">
+        <x:v>13.7</x:v>
+      </x:c>
+      <x:c r="J366" t="n">
+        <x:v>65.2</x:v>
+      </x:c>
+      <x:c r="K366"/>
+      <x:c r="L366" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M366"/>
+      <x:c r="N366" s="29"/>
+      <x:c r="O366" t="str">
+        <x:v>אגוז שלם (2 חצאים, כ-4 גרם)</x:v>
+      </x:c>
+      <x:c r="P366" t="str">
+        <x:v>ממתין לבדיקה</x:v>
+      </x:c>
+      <x:c r="Q366" t="str">
+        <x:v>ערכים ל-100 גרם שנמסרו על ידי המשתמש; סיבים תזונתיים: כ-6.7 גרם. חצי אגוז (כ-2 גרם): כ-13 קלוריות; חופן של כ-30 גרם: כ-196 קלוריות.</x:v>
+      </x:c>
+      <x:c r="R366"/>
+      <x:c r="S366" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="T366" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="U366" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="367">
+      <x:c r="A367" t="str">
+        <x:v>roasted-salted-almonds</x:v>
+      </x:c>
+      <x:c r="B367" t="str">
+        <x:v>אגוזים וזרעים</x:v>
+      </x:c>
+      <x:c r="C367" t="str">
+        <x:v>שקדים קלויים ומלוחים</x:v>
+      </x:c>
+      <x:c r="D367"/>
+      <x:c r="E367"/>
+      <x:c r="F367" t="str">
+        <x:v>יחידה</x:v>
+      </x:c>
+      <x:c r="G367" t="n">
+        <x:v>613</x:v>
+      </x:c>
+      <x:c r="H367" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="I367" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J367" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="K367" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L367" t="n">
+        <x:v>650</x:v>
+      </x:c>
+      <x:c r="M367"/>
+      <x:c r="N367" s="29"/>
+      <x:c r="O367" t="str">
+        <x:v>שקד אחד (כ-1.2 גרם)</x:v>
+      </x:c>
+      <x:c r="P367" t="str">
+        <x:v>ממתין לבדיקה</x:v>
+      </x:c>
+      <x:c r="Q367" t="str">
+        <x:v>ערכים ל-100 גרם שנמסרו על ידי המשתמש; שומן רווי: 4 גרם; סיבים תזונתיים: כ-3.5 גרם. חופן של כ-30 גרם: כ-184 קלוריות.</x:v>
+      </x:c>
+      <x:c r="R367"/>
+      <x:c r="S367" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="T367" t="n">
+        <x:v>7.3</x:v>
+      </x:c>
+      <x:c r="U367" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:R1"/>
@@ -22295,7 +22403,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f4d7261ae30498d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R831a795cd4e247b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Show walnuts and almonds per 100g
</commit_message>
<xml_diff>
--- a/data/source/foods.xlsx
+++ b/data/source/foods.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="Rb0aab3d189e14df2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="בלוק 1 - מוצרי חלב" sheetId="1" r:id="R00e7b75fff224d9d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22290,9 +22290,7 @@
       </x:c>
       <x:c r="D366"/>
       <x:c r="E366"/>
-      <x:c r="F366" t="str">
-        <x:v>יחידה</x:v>
-      </x:c>
+      <x:c r="F366"/>
       <x:c r="G366" t="n">
         <x:v>654</x:v>
       </x:c>
@@ -22312,24 +22310,18 @@
       <x:c r="M366"/>
       <x:c r="N366" s="29"/>
       <x:c r="O366" t="str">
-        <x:v>אגוז שלם (2 חצאים, כ-4 גרם)</x:v>
+        <x:v>ל-100 גרם</x:v>
       </x:c>
       <x:c r="P366" t="str">
         <x:v>ממתין לבדיקה</x:v>
       </x:c>
       <x:c r="Q366" t="str">
-        <x:v>ערכים ל-100 גרם שנמסרו על ידי המשתמש; סיבים תזונתיים: כ-6.7 גרם. חצי אגוז (כ-2 גרם): כ-13 קלוריות; חופן של כ-30 גרם: כ-196 קלוריות.</x:v>
+        <x:v>ערכים ל-100 גרם שנמסרו על ידי המשתמש; סיבים תזונתיים: כ-6.7 גרם.</x:v>
       </x:c>
       <x:c r="R366"/>
-      <x:c r="S366" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="T366" t="n">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="U366" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="S366"/>
+      <x:c r="T366"/>
+      <x:c r="U366"/>
     </x:row>
     <x:row r="367">
       <x:c r="A367" t="str">
@@ -22343,9 +22335,7 @@
       </x:c>
       <x:c r="D367"/>
       <x:c r="E367"/>
-      <x:c r="F367" t="str">
-        <x:v>יחידה</x:v>
-      </x:c>
+      <x:c r="F367"/>
       <x:c r="G367" t="n">
         <x:v>613</x:v>
       </x:c>
@@ -22367,24 +22357,18 @@
       <x:c r="M367"/>
       <x:c r="N367" s="29"/>
       <x:c r="O367" t="str">
-        <x:v>שקד אחד (כ-1.2 גרם)</x:v>
+        <x:v>ל-100 גרם</x:v>
       </x:c>
       <x:c r="P367" t="str">
         <x:v>ממתין לבדיקה</x:v>
       </x:c>
       <x:c r="Q367" t="str">
-        <x:v>ערכים ל-100 גרם שנמסרו על ידי המשתמש; שומן רווי: 4 גרם; סיבים תזונתיים: כ-3.5 גרם. חופן של כ-30 גרם: כ-184 קלוריות.</x:v>
+        <x:v>ערכים ל-100 גרם שנמסרו על ידי המשתמש; שומן רווי: 4 גרם; סיבים תזונתיים: כ-3.5 גרם.</x:v>
       </x:c>
       <x:c r="R367"/>
-      <x:c r="S367" t="n">
-        <x:v>1.2</x:v>
-      </x:c>
-      <x:c r="T367" t="n">
-        <x:v>7.3</x:v>
-      </x:c>
-      <x:c r="U367" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="S367"/>
+      <x:c r="T367"/>
+      <x:c r="U367"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -22403,7 +22387,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R831a795cd4e247b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a79ff6bd69e469c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>